<commit_message>
refactor(rates): load rates.json from skill root instead of scripts/
</commit_message>
<xml_diff>
--- a/.claude/skills/weekly-hours-report/scripts/cache/sheet-Jul-2026.xlsx
+++ b/.claude/skills/weekly-hours-report/scripts/cache/sheet-Jul-2026.xlsx
@@ -2762,42 +2762,42 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>1</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>0</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -2886,7 +2886,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -3038,7 +3038,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -3507,6 +3507,11 @@
           <t>PTO</t>
         </is>
       </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>ML(PA)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3563,7 +3568,7 @@
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>Celeste Dominguez</t>
+          <t>Celeste Dominguez 9-10</t>
         </is>
       </c>
     </row>
@@ -3634,6 +3639,11 @@
           <t>H</t>
         </is>
       </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>ML(PA)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3781,7 +3791,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>ML(PA)</t>
+          <t>ML</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3813,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>PTO(PA)</t>
+          <t>PTO</t>
         </is>
       </c>
     </row>
@@ -3872,6 +3882,11 @@
           <t>PTO</t>
         </is>
       </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>ML(PA)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4004,6 +4019,11 @@
           <t>H</t>
         </is>
       </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ML(PA)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4343,7 +4363,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>ML(PA)</t>
+          <t>ML</t>
         </is>
       </c>
     </row>
@@ -4754,6 +4774,11 @@
         </is>
       </c>
       <c r="L62" t="inlineStr">
+        <is>
+          <t>PTO(PA)</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
         <is>
           <t>PTO(PA)</t>
         </is>

</xml_diff>